<commit_message>
Traverse & Level 2.1: updated manual, screens and samples
- User manual (PowerPoint and PDF, 41 slides): new section 4, Angles & distances:
  the field book, side shots and closing leg, the field book result, angles and
  side shots, least squares settings and results, Qatar National Grid, and the
  PDF / CSV / Google Earth exports. Contents, intro, simulator and PDF slides
  updated; a second quick reference for choosing the input.
- Product page: version 2.1, three new screens (field book, least squares,
  Qatar National Grid), retaken traverse screens, new field book samples
  (CSV, PDF report, KML) and a Field book sheet in sample-data.xlsx.
- App: angle and distance cells in the field book are wide enough for
  DDD.MMSS values; side-shot labels on the plan and in the PDF sketch sit
  beyond the point so they no longer cover the station's label.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016D4TXLBZZoVtCPNFo121Mg
</commit_message>
<xml_diff>
--- a/public/traverse/samples/sample-data.xlsx
+++ b/public/traverse/samples/sample-data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traverse" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Level book" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field book" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -80,6 +81,11 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -747,4 +753,283 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Field book (angles and distances, closed loop on CP-01 with levels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Choose Angles &amp; distances. Known points: CP-01 228450.312 / 441203.845 · CP-02 228912.640 / 441655.118 · closing CP-01 (loop). Settings: angle turned from the backsight, DDD.MMSS, clockwise, Levels ticked, station level 4.215. Copy rows 4 to 11 (header included) and paste into the first Side cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Closing leg (row C): angle 130.2740, distance 288.697, ht diff -0.523 · closing angle at CP-01 onto CP-02: 23.1021</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Angle</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Ht diff</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>81.3127</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>316.630</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>0.646</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>TS-01</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Nail in kerb</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Side shot</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>312.4500</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>42.315</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-0.212</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>MH-01</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Manhole cover</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>124.3129</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>308.240</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>0.584</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>TS-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>125.5354</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>308.364</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>0.566</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>TS-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Side shot</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>201.1530</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>27.904</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>0.118</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>LP-01</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Lamp post</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>104.5917</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>293.903</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-0.802</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>TS-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>129.2554</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>294.528</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>-0.478</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>TS-05</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>